<commit_message>
Remove workbook control language and strengthen AI gate
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R67026c17f568424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R4e700978918f4691"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -544,27 +544,11 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
-      <x:c r="A17" s="22" t="str">
+      <x:c r="A17" s="24" t="str">
         <x:v>完成条件</x:v>
       </x:c>
-      <x:c r="B17" s="23" t="str">
+      <x:c r="B17" s="25" t="str">
         <x:v>npm run process:hls返回0，五个目标路径可读，四份报告以asset_id和profile闭合</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="48" customHeight="1">
-      <x:c r="A18" s="22" t="str">
-        <x:v>可验证点</x:v>
-      </x:c>
-      <x:c r="B18" s="23" t="str">
-        <x:v>master引用、profile映射、片段配对、缺片、时长、编码、码率范围、梯度、主原因、动作、来源路径和排序</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="33" customHeight="1">
-      <x:c r="A19" s="24" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
-      </x:c>
-      <x:c r="B19" s="25" t="str">
-        <x:v>函数拆分、变量名、注释、内部对象、临时数组、CSV必要引号及LF或CRLF行尾</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>